<commit_message>
new tasks and exercise for excel in latest class and sql task to practise in integrated tasks. 90% complete.
</commit_message>
<xml_diff>
--- a/Excel classes/class 23 Tasks/Sales Data.xlsx
+++ b/Excel classes/class 23 Tasks/Sales Data.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ueducation-my.sharepoint.com/personal/devashish_das_upgrad_com/Documents/Desktop/Revision/Excel/mock_task/sales_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddh\Desktop\Codepro\Upgrad classes\Excel classes\class 23 Tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{492D46BF-4D26-4C3F-A908-615E8C3F7E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC489F06-D6D8-4AF9-B139-2D611D34CDA8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F147864-FD60-4A07-A670-7A7F13A1B1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BA44CE9A-29A7-48B7-8579-F97E326B652B}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="15084" windowHeight="13056" xr2:uid="{BA44CE9A-29A7-48B7-8579-F97E326B652B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -130,13 +143,16 @@
     <t>C014</t>
   </si>
   <si>
-    <t>l</t>
+    <t>Month</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -614,9 +630,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -662,7 +682,17 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -673,6 +703,29 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5EA72B5-1CD8-499E-B03A-C1ACB6839ED6}" name="Table1" displayName="Table1" ref="A1:I15" totalsRowShown="0">
+  <autoFilter ref="A1:I15" xr:uid="{D5EA72B5-1CD8-499E-B03A-C1ACB6839ED6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H15">
+    <sortCondition ref="B2:B15"/>
+  </sortState>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{22FA97F7-726D-4F69-BB2B-AE607D329968}" name="OrderID"/>
+    <tableColumn id="2" xr3:uid="{EE75F02F-A741-4510-B3F2-2A715A90D763}" name="OrderDate" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{015214F9-5B6C-4DDA-AA1E-469AE8137BD9}" name="Product"/>
+    <tableColumn id="4" xr3:uid="{6770E9F5-5A28-49B3-9C8D-1715A6FCF6E3}" name="Category"/>
+    <tableColumn id="5" xr3:uid="{A717B77A-ED64-4AF9-A290-0B29F90ECE9A}" name="Region"/>
+    <tableColumn id="6" xr3:uid="{2629213B-EB85-4157-BD22-7127BB8B1D8B}" name="Amount" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{6148150A-2AAD-42A8-B672-E0F096490EA8}" name="Quantity"/>
+    <tableColumn id="8" xr3:uid="{FC3003A8-437A-4423-8E94-8A92E1D1D681}" name="CustomerID"/>
+    <tableColumn id="9" xr3:uid="{55668C60-BEF3-4298-BF2C-25D9D7462BBC}" name="Month" dataDxfId="0">
+      <calculatedColumnFormula>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -992,39 +1045,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14154331-1AED-4926-85A2-566CAE8414C6}">
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7265625" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="10" max="10" width="8.21875" customWidth="1"/>
+    <col min="11" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="3" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1040,7 +1104,7 @@
       <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>1200</v>
       </c>
       <c r="G2">
@@ -1049,8 +1113,12 @@
       <c r="H2" t="s">
         <v>11</v>
       </c>
+      <c r="I2" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Jan</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -1066,7 +1134,7 @@
       <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>50</v>
       </c>
       <c r="G3">
@@ -1075,8 +1143,16 @@
       <c r="H3" t="s">
         <v>14</v>
       </c>
+      <c r="I3" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Feb</v>
+      </c>
+      <c r="L3">
+        <f>COUNT(A2:A15)</f>
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1092,7 +1168,7 @@
       <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>300</v>
       </c>
       <c r="G4">
@@ -1101,8 +1177,16 @@
       <c r="H4" t="s">
         <v>18</v>
       </c>
+      <c r="I4" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Mar</v>
+      </c>
+      <c r="L4">
+        <f>MAX(F2:F15)</f>
+        <v>1200</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1118,7 +1202,7 @@
       <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>400</v>
       </c>
       <c r="G5">
@@ -1127,8 +1211,12 @@
       <c r="H5" t="s">
         <v>21</v>
       </c>
+      <c r="I5" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Apr</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1144,7 +1232,7 @@
       <c r="E6" t="s">
         <v>10</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>150</v>
       </c>
       <c r="G6">
@@ -1153,8 +1241,12 @@
       <c r="H6" t="s">
         <v>23</v>
       </c>
+      <c r="I6" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>May</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1170,7 +1262,7 @@
       <c r="E7" t="s">
         <v>13</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>80</v>
       </c>
       <c r="G7">
@@ -1179,8 +1271,16 @@
       <c r="H7" t="s">
         <v>25</v>
       </c>
+      <c r="I7" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Jun</v>
+      </c>
+      <c r="L7">
+        <f>SUM(Table1[Quantity])</f>
+        <v>19</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1196,7 +1296,7 @@
       <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <v>600</v>
       </c>
       <c r="G8">
@@ -1205,8 +1305,12 @@
       <c r="H8" t="s">
         <v>27</v>
       </c>
+      <c r="I8" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Jul</v>
+      </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1222,7 +1326,7 @@
       <c r="E9" t="s">
         <v>20</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <v>1000</v>
       </c>
       <c r="G9">
@@ -1231,8 +1335,16 @@
       <c r="H9" t="s">
         <v>29</v>
       </c>
+      <c r="I9" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Aug</v>
+      </c>
+      <c r="L9">
+        <f>AVERAGE(Table1[Amount])</f>
+        <v>426.78571428571428</v>
+      </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1248,7 +1360,7 @@
       <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <v>1100</v>
       </c>
       <c r="G10">
@@ -1257,8 +1369,16 @@
       <c r="H10" t="s">
         <v>30</v>
       </c>
+      <c r="I10" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Sep</v>
+      </c>
+      <c r="L10" s="2">
+        <f>SUM(Table1[Amount])</f>
+        <v>5975</v>
+      </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1274,7 +1394,7 @@
       <c r="E11" t="s">
         <v>13</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
         <v>45</v>
       </c>
       <c r="G11">
@@ -1283,8 +1403,16 @@
       <c r="H11" t="s">
         <v>31</v>
       </c>
+      <c r="I11" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Oct</v>
+      </c>
+      <c r="L11" t="e">
+        <f>_xlfn.MODE.SNGL(Table1[Product])</f>
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1300,7 +1428,7 @@
       <c r="E12" t="s">
         <v>17</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="2">
         <v>350</v>
       </c>
       <c r="G12">
@@ -1309,8 +1437,16 @@
       <c r="H12" t="s">
         <v>32</v>
       </c>
+      <c r="I12" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Nov</v>
+      </c>
+      <c r="L12">
+        <f>COUNTIF(Table1[Region],"north")</f>
+        <v>4</v>
+      </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1326,7 +1462,7 @@
       <c r="E13" t="s">
         <v>20</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="2">
         <v>450</v>
       </c>
       <c r="G13">
@@ -1335,8 +1471,12 @@
       <c r="H13" t="s">
         <v>33</v>
       </c>
+      <c r="I13" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Dec</v>
+      </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1013</v>
       </c>
@@ -1352,7 +1492,7 @@
       <c r="E14" t="s">
         <v>10</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="2">
         <v>160</v>
       </c>
       <c r="G14">
@@ -1361,8 +1501,12 @@
       <c r="H14" t="s">
         <v>34</v>
       </c>
+      <c r="I14" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Jan</v>
+      </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1014</v>
       </c>
@@ -1378,7 +1522,7 @@
       <c r="E15" t="s">
         <v>13</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="2">
         <v>90</v>
       </c>
       <c r="G15">
@@ -1387,18 +1531,15 @@
       <c r="H15" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D18" t="s">
-        <v>36</v>
+      <c r="I15" t="str">
+        <f>TEXT(Table1[[#This Row],[OrderDate]],"mmm")</f>
+        <v>Feb</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>